<commit_message>
Adds worksheet metadata parsing (not contents yet)
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9BC055B-8B20-464B-8590-2607DCBEF424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89D9595-6C20-47B2-8EE9-CCD28720518A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17016" yWindow="9144" windowWidth="14496" windowHeight="11976" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="9516" yWindow="10032" windowWidth="26892" windowHeight="11976" activeTab="1" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Items" sheetId="1" r:id="rId1"/>
+    <sheet name="Others" sheetId="3" r:id="rId2"/>
+    <sheet name="Monsters" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>item</t>
   </si>
@@ -72,13 +74,31 @@
   </si>
   <si>
     <t>staff of destruction</t>
+  </si>
+  <si>
+    <t>monster</t>
+  </si>
+  <si>
+    <t>hp</t>
+  </si>
+  <si>
+    <t>spd</t>
+  </si>
+  <si>
+    <t>slime</t>
+  </si>
+  <si>
+    <t>spider</t>
+  </si>
+  <si>
+    <t>bat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,13 +106,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Abadi ExtraLight"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -107,8 +155,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,29 +504,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{668D3AAD-1C86-48AC-9E87-A54614A0E569}">
   <dimension ref="B2:G8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="5.21875" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
+    <row r="2" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B3">
+    <row r="3" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="5">
         <v>1</v>
       </c>
       <c r="C3" t="s">
@@ -483,12 +546,12 @@
         <f>IF(E3&lt;4,2*E3,1.5*E3)</f>
         <v>6.3000000000000007</v>
       </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4">
+      <c r="G3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
       <c r="C4" t="s">
@@ -501,13 +564,13 @@
         <f t="shared" ref="F4:F8" si="0">IF(E4&lt;4,2*E4,1.5*E4)</f>
         <v>0</v>
       </c>
-      <c r="G4" t="b">
+      <c r="G4" s="3" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B5">
+    <row r="5" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -523,13 +586,13 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="G5" t="b">
+      <c r="G5" s="3" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B6">
+    <row r="6" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="5">
         <v>4</v>
       </c>
       <c r="C6" t="s">
@@ -545,13 +608,13 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="G6" t="b">
+      <c r="G6" s="3" t="b">
         <f>FALSE</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7">
+    <row r="7" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="5">
         <v>5</v>
       </c>
       <c r="C7" t="str">
@@ -568,13 +631,13 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G7" t="b">
+      <c r="G7" s="3" t="b">
         <f>TRUE</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8">
+    <row r="8" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="5">
         <v>6</v>
       </c>
       <c r="C8" t="s">
@@ -587,9 +650,84 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="G8" t="b">
+      <c r="G8" s="3" t="b">
         <f>TRUE</f>
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBAE049A-BB92-4092-98D0-27C0B6A0646A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35E7FE3-F747-44A2-B918-3E58803B642A}">
+  <dimension ref="C5:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="5" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>7</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds foundations of cell parsing from a sheet
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89D9595-6C20-47B2-8EE9-CCD28720518A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0DD029-078B-4584-B30F-E065C9030DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9516" yWindow="10032" windowWidth="26892" windowHeight="11976" activeTab="1" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="9516" yWindow="10032" windowWidth="26892" windowHeight="11976" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -543,8 +543,8 @@
         <v>4.2</v>
       </c>
       <c r="F3">
-        <f>IF(E3&lt;4,2*E3,1.5*E3)</f>
-        <v>6.3000000000000007</v>
+        <f>E3*2</f>
+        <v>8.4</v>
       </c>
       <c r="G3" s="3">
         <v>1</v>
@@ -561,7 +561,7 @@
         <v>2</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4:F8" si="0">IF(E4&lt;4,2*E4,1.5*E4)</f>
+        <f t="shared" ref="F4:F8" si="0">E4*2</f>
         <v>0</v>
       </c>
       <c r="G4" s="3" t="b">
@@ -606,7 +606,7 @@
       </c>
       <c r="F6">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G6" s="3" t="b">
         <f>FALSE</f>

</xml_diff>

<commit_message>
Fixes a bug with formula parsing and tests a bigger synthetic data XLSX
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0DD029-078B-4584-B30F-E065C9030DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A56ACA-07F8-4BBC-AD27-050B8FF79414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9516" yWindow="10032" windowWidth="26892" windowHeight="11976" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="-90" yWindow="3390" windowWidth="25690" windowHeight="11890" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -643,12 +643,12 @@
       <c r="C8" t="s">
         <v>4</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>3</v>
       </c>
       <c r="F8">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>IF(E8=3,1,0)</f>
+        <v>1</v>
       </c>
       <c r="G8" s="3" t="b">
         <f>TRUE</f>

</xml_diff>

<commit_message>
Adds HTML entity unescaping to values and formulas
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A56ACA-07F8-4BBC-AD27-050B8FF79414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE4E599-E897-49E5-A924-5B7C66B43E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="3390" windowWidth="25690" windowHeight="11890" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -507,6 +507,7 @@
   <cols>
     <col min="2" max="2" width="5.21875" customWidth="1"/>
     <col min="3" max="3" width="26.5546875" customWidth="1"/>
+    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -599,14 +600,14 @@
         <v>10</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E6">
         <v>8</v>
       </c>
-      <c r="F6">
-        <f t="shared" si="0"/>
-        <v>16</v>
+      <c r="F6" t="str">
+        <f ca="1">IF(AND(E6&gt;2,D6&lt;1), "&amp;"&amp;TEXT(RAND(),"#.###"), "M&amp;Ms are "&amp;TEXT(2.1,"#"))</f>
+        <v>&amp;.046</v>
       </c>
       <c r="G6" s="3" t="b">
         <f>FALSE</f>
@@ -627,9 +628,9 @@
       <c r="E7">
         <v>2</v>
       </c>
-      <c r="F7">
-        <f t="shared" si="0"/>
-        <v>4</v>
+      <c r="F7" t="str">
+        <f ca="1">IF(AND(E7&gt;2,D7&lt;1), "&amp;"&amp;TEXT(RAND(),"#.###"), "M&amp;Ms are "&amp;TEXT(2.1,"#"))</f>
+        <v>M&amp;Ms are 2</v>
       </c>
       <c r="G7" s="3" t="b">
         <f>TRUE</f>

</xml_diff>

<commit_message>
Implements basic field schema validation and creates the table
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE4E599-E897-49E5-A924-5B7C66B43E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487C918F-BC07-4837-AEB5-7877AC743D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>item</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>bat</t>
+  </si>
+  <si>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -562,8 +565,7 @@
         <v>2</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4:F8" si="0">E4*2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="3" t="b">
         <f>TRUE</f>
@@ -584,12 +586,11 @@
         <v>3</v>
       </c>
       <c r="F5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F4:F8" si="0">E5*2</f>
         <v>6</v>
       </c>
-      <c r="G5" s="3" t="b">
-        <f>TRUE</f>
-        <v>1</v>
+      <c r="G5" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -605,9 +606,8 @@
       <c r="E6">
         <v>8</v>
       </c>
-      <c r="F6" t="str">
-        <f ca="1">IF(AND(E6&gt;2,D6&lt;1), "&amp;"&amp;TEXT(RAND(),"#.###"), "M&amp;Ms are "&amp;TEXT(2.1,"#"))</f>
-        <v>&amp;.046</v>
+      <c r="F6">
+        <v>4.25</v>
       </c>
       <c r="G6" s="3" t="b">
         <f>FALSE</f>
@@ -628,12 +628,10 @@
       <c r="E7">
         <v>2</v>
       </c>
-      <c r="F7" t="str">
-        <f ca="1">IF(AND(E7&gt;2,D7&lt;1), "&amp;"&amp;TEXT(RAND(),"#.###"), "M&amp;Ms are "&amp;TEXT(2.1,"#"))</f>
-        <v>M&amp;Ms are 2</v>
+      <c r="F7">
+        <v>8.1999999999999993</v>
       </c>
       <c r="G7" s="3" t="b">
-        <f>TRUE</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixes management of blank values
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487C918F-BC07-4837-AEB5-7877AC743D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8377970D-2CE2-4962-99DB-67C79D0ABB80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" activeTab="2" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -717,16 +717,13 @@
     </row>
     <row r="8" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds named ranges support
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7ADD952-5B44-4688-BDF8-A66C67D5A1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADAA1C9-FBA5-4EEC-BDE6-4E08F03F3361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
@@ -17,6 +17,9 @@
     <sheet name="Others" sheetId="3" r:id="rId2"/>
     <sheet name="Monsters" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="my_named">Items!$C$5:$F$7</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">

</xml_diff>

<commit_message>
Adds ID uniqueness check
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADAA1C9-FBA5-4EEC-BDE6-4E08F03F3361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B42BE8A-8EF1-4D05-9364-35CD5CABA1DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
@@ -577,7 +577,7 @@
     </row>
     <row r="5" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Adds foreign key validation
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873C78C3-752B-4288-BCA5-34C6A7A529C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF7F8B9-3FF3-4C8B-BD0C-BE70B1E5F746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
@@ -19,6 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="my_named">Items!$C$5:$F$7</definedName>
+    <definedName name="powers">Items!$M$2:$O$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>item</t>
   </si>
@@ -98,6 +99,39 @@
   </si>
   <si>
     <t>Y</t>
+  </si>
+  <si>
+    <t>power</t>
+  </si>
+  <si>
+    <t>power_id</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>p1</t>
+  </si>
+  <si>
+    <t>p2</t>
+  </si>
+  <si>
+    <t>p3</t>
+  </si>
+  <si>
+    <t>first level</t>
+  </si>
+  <si>
+    <t>third level</t>
+  </si>
+  <si>
+    <t>second level</t>
+  </si>
+  <si>
+    <t>p4</t>
   </si>
 </sst>
 </file>
@@ -508,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{668D3AAD-1C86-48AC-9E87-A54614A0E569}">
-  <dimension ref="B2:G8"/>
+  <dimension ref="B2:O8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="5.21875" customWidth="1"/>
@@ -516,7 +550,7 @@
     <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -535,8 +569,20 @@
       <c r="G2" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5">
         <v>1</v>
       </c>
@@ -556,8 +602,17 @@
       <c r="G3" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5">
         <v>2</v>
       </c>
@@ -574,8 +629,20 @@
         <f>TRUE</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="M4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5">
         <v>3</v>
       </c>
@@ -595,8 +662,17 @@
       <c r="G5" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M5" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" t="s">
+        <v>26</v>
+      </c>
+      <c r="O5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="5">
         <v>4</v>
       </c>
@@ -616,8 +692,11 @@
         <f>FALSE</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="5">
         <v>5</v>
       </c>
@@ -637,8 +716,11 @@
       <c r="G7" s="3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="5">
         <v>6</v>
       </c>
@@ -658,6 +740,9 @@
       <c r="G8" s="3" t="b">
         <f>TRUE</f>
         <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improves schema parameter validations
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF7F8B9-3FF3-4C8B-BD0C-BE70B1E5F746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86280B9-BD2D-4CE4-A6A5-F8BA9FFAB69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>item</t>
   </si>
@@ -129,9 +129,6 @@
   </si>
   <si>
     <t>second level</t>
-  </si>
-  <si>
-    <t>p4</t>
   </si>
 </sst>
 </file>
@@ -630,7 +627,7 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="M4" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
Improves schema validation for FK
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86280B9-BD2D-4CE4-A6A5-F8BA9FFAB69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888C0DAC-F158-4328-9EBC-7061522EA3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" activeTab="2" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>item</t>
   </si>
@@ -129,6 +129,27 @@
   </si>
   <si>
     <t>second level</t>
+  </si>
+  <si>
+    <t>configurable</t>
+  </si>
+  <si>
+    <t>max_value</t>
+  </si>
+  <si>
+    <t>min_value</t>
+  </si>
+  <si>
+    <t>filename</t>
+  </si>
+  <si>
+    <t>C:\Users\biyec\AppData\Local\Spread</t>
+  </si>
+  <si>
+    <t>formula</t>
+  </si>
+  <si>
+    <t>=if(x&lt;=2, "test", 'my god'</t>
   </si>
 </sst>
 </file>
@@ -192,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -205,6 +226,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,10 +780,37 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35E7FE3-F747-44A2-B918-3E58803B642A}">
-  <dimension ref="C5:F8"/>
+  <dimension ref="C2:K8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="10" max="10" width="14.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="5" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="J2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="J3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3">
+        <v>513.41999999999996</v>
+      </c>
+    </row>
+    <row r="4" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="J4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4">
+        <v>12.5235</v>
+      </c>
+    </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
@@ -774,8 +823,14 @@
       <c r="F5" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="J5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>12</v>
       </c>
@@ -788,8 +843,14 @@
       <c r="F6">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="J6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>13</v>
       </c>
@@ -803,7 +864,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Adds JSON bundle reading and writing
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888C0DAC-F158-4328-9EBC-7061522EA3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06320B1-ACCB-4B57-875B-5F337650C033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14328" yWindow="13548" windowWidth="22416" windowHeight="9984" activeTab="2" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="5940" yWindow="8736" windowWidth="22332" windowHeight="9888" activeTab="2" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>item</t>
   </si>
@@ -129,27 +129,6 @@
   </si>
   <si>
     <t>second level</t>
-  </si>
-  <si>
-    <t>configurable</t>
-  </si>
-  <si>
-    <t>max_value</t>
-  </si>
-  <si>
-    <t>min_value</t>
-  </si>
-  <si>
-    <t>filename</t>
-  </si>
-  <si>
-    <t>C:\Users\biyec\AppData\Local\Spread</t>
-  </si>
-  <si>
-    <t>formula</t>
-  </si>
-  <si>
-    <t>=if(x&lt;=2, "test", 'my god'</t>
   </si>
 </sst>
 </file>
@@ -780,37 +759,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35E7FE3-F747-44A2-B918-3E58803B642A}">
-  <dimension ref="C2:K8"/>
+  <dimension ref="C5:L8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="10" max="10" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="J2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="J3" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3">
-        <v>513.41999999999996</v>
-      </c>
-    </row>
-    <row r="4" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="J4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4">
-        <v>12.5235</v>
-      </c>
-    </row>
-    <row r="5" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
@@ -823,14 +778,8 @@
       <c r="F5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J5" t="s">
-        <v>31</v>
-      </c>
-      <c r="K5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="3:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>12</v>
       </c>
@@ -843,14 +792,10 @@
       <c r="F6">
         <v>3</v>
       </c>
-      <c r="J6" t="s">
-        <v>33</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+    </row>
+    <row r="7" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>13</v>
       </c>
@@ -864,7 +809,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="3:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Adds date inferring from Spread_Num (no timezone management)
</commit_message>
<xml_diff>
--- a/datafiles/Test.xlsx
+++ b/datafiles/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biyec\GameMakerProjects\Other Mine\Spread\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06320B1-ACCB-4B57-875B-5F337650C033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04970742-0B77-49B4-8736-DA590A643875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5940" yWindow="8736" windowWidth="22332" windowHeight="9888" activeTab="2" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
+    <workbookView xWindow="144" yWindow="0" windowWidth="25644" windowHeight="15372" xr2:uid="{4F78AFE7-D6EA-4F35-AA43-EEE94C22C300}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>item</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>second level</t>
+  </si>
+  <si>
+    <t>dt</t>
   </si>
 </sst>
 </file>
@@ -192,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -206,6 +209,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,6 +550,7 @@
     <col min="2" max="2" width="5.21875" customWidth="1"/>
     <col min="3" max="3" width="26.5546875" customWidth="1"/>
     <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -570,6 +575,9 @@
       <c r="H2" s="4" t="s">
         <v>18</v>
       </c>
+      <c r="I2" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="M2" t="s">
         <v>19</v>
       </c>
@@ -600,6 +608,9 @@
       <c r="G3" s="3">
         <v>1</v>
       </c>
+      <c r="I3" s="7">
+        <v>76310</v>
+      </c>
       <c r="M3" t="s">
         <v>22</v>
       </c>
@@ -630,6 +641,9 @@
       <c r="H4" t="s">
         <v>24</v>
       </c>
+      <c r="I4" s="7">
+        <v>18638</v>
+      </c>
       <c r="M4" t="s">
         <v>23</v>
       </c>
@@ -654,11 +668,14 @@
         <v>3</v>
       </c>
       <c r="F5">
-        <f t="shared" ref="F4:F8" si="0">E5*2</f>
+        <f t="shared" ref="F5" si="0">E5*2</f>
         <v>6</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>17</v>
+      </c>
+      <c r="I5" s="7">
+        <v>26736</v>
       </c>
       <c r="M5" t="s">
         <v>24</v>
@@ -693,6 +710,9 @@
       <c r="H6" t="s">
         <v>23</v>
       </c>
+      <c r="I6" s="7">
+        <v>54799</v>
+      </c>
     </row>
     <row r="7" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="5">
@@ -717,6 +737,9 @@
       <c r="H7" t="s">
         <v>24</v>
       </c>
+      <c r="I7" s="7">
+        <v>79269</v>
+      </c>
     </row>
     <row r="8" spans="2:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="5">
@@ -741,6 +764,9 @@
       </c>
       <c r="H8" t="s">
         <v>22</v>
+      </c>
+      <c r="I8" s="7">
+        <v>98017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>